<commit_message>
Expand eval package: formulas under 80% typed, PO lines, inventory variance
- Corrected Register / Source Ledger / Exception Register / Ledger Reconciliation
  now use XLOOKUP and derived formulas with OOXML caches (typed ratio ~78.9%)
- Source Inventory sheet added for register lookups
- hardware_purchase_orders.csv expanded to asset-level line items with uneven
  PO batch sizes (1–9 assets)
- it_asset_inventory.xlsx: uneven categories and 21 hardware models
- check_outputs already gates on Yanou filename + OOXML type
- Revision 2.18

Co-authored-by: efokou <EtienneFokou-E18560@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/it_asset_inventory.xlsx
+++ b/it_asset_inventory.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset Register" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Asset Register" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -506,12 +506,12 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14</t>
+          <t>HP EliteBook 840 G10</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -557,12 +557,12 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Microsoft Surface Laptop 5</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -608,12 +608,12 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Lenovo ThinkPad X1 Carbon</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -659,12 +659,12 @@
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Lenovo ThinkPad T14</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -761,12 +761,12 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Dell Latitude 7440</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
@@ -812,12 +812,12 @@
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>HP EliteBook 840 G10</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
@@ -863,12 +863,12 @@
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Samsung ViewFinity S8</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -914,12 +914,12 @@
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Dell Latitude 7440</t>
+          <t>BenQ PD2705U</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -1016,12 +1016,12 @@
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>LG UltraFine 27MD5KL</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -1067,12 +1067,12 @@
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Samsung ViewFinity S8</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
@@ -1118,12 +1118,12 @@
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14</t>
+          <t>BenQ PD2705U</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Dell P2422H</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -1220,12 +1220,12 @@
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Dell U2723QE</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
@@ -1271,12 +1271,12 @@
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>LG UltraFine 27MD5KL</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -1322,12 +1322,12 @@
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>MacBook Pro 14</t>
+          <t>Samsung ViewFinity S8</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>BenQ PD2705U</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Dell P2422H</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
@@ -1475,12 +1475,12 @@
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>LG UltraFine 27MD5KL</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
@@ -1526,12 +1526,12 @@
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Dell Latitude 7440</t>
+          <t>Samsung ViewFinity S8</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>BenQ PD2705U</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
@@ -1628,12 +1628,12 @@
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Dell P2422H</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
@@ -1679,12 +1679,12 @@
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Dell U2723QE</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -1730,12 +1730,12 @@
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14</t>
+          <t>LG UltraFine 27MD5KL</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Samsung ViewFinity S8</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -1832,12 +1832,12 @@
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>BenQ PD2705U</t>
         </is>
       </c>
       <c r="E31" s="12" t="inlineStr">
@@ -1883,12 +1883,12 @@
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Dell P2422H</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -1934,12 +1934,12 @@
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D33" s="12" t="inlineStr">
         <is>
-          <t>MacBook Pro 14</t>
+          <t>Dell U2723QE</t>
         </is>
       </c>
       <c r="E33" s="12" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="D34" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Samsung ViewFinity S8</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -2036,12 +2036,12 @@
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D35" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>BenQ PD2705U</t>
         </is>
       </c>
       <c r="E35" s="12" t="inlineStr">
@@ -2087,12 +2087,12 @@
       </c>
       <c r="C36" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Dell P2422H</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
@@ -2138,12 +2138,12 @@
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D37" s="12" t="inlineStr">
         <is>
-          <t>Dell Latitude 7440</t>
+          <t>Dell U2723QE</t>
         </is>
       </c>
       <c r="E37" s="12" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="D38" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>LG UltraFine 27MD5KL</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -2240,12 +2240,12 @@
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="D39" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Samsung ViewFinity S8</t>
         </is>
       </c>
       <c r="E39" s="12" t="inlineStr">
@@ -2291,12 +2291,12 @@
       </c>
       <c r="C40" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Samsung Galaxy S23 FE</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -2342,12 +2342,12 @@
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D41" s="12" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14</t>
+          <t>iPhone 14</t>
         </is>
       </c>
       <c r="E41" s="12" t="inlineStr">
@@ -2393,12 +2393,12 @@
       </c>
       <c r="C42" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Samsung Galaxy S24</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="D43" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>iPhone 15</t>
         </is>
       </c>
       <c r="E43" s="12" t="inlineStr">
@@ -2495,12 +2495,12 @@
       </c>
       <c r="C44" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Samsung Galaxy S23 FE</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -2546,12 +2546,12 @@
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D45" s="12" t="inlineStr">
         <is>
-          <t>MacBook Pro 14</t>
+          <t>iPhone 14</t>
         </is>
       </c>
       <c r="E45" s="12" t="inlineStr">
@@ -2597,12 +2597,12 @@
       </c>
       <c r="C46" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Samsung Galaxy S24</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
@@ -2653,7 +2653,7 @@
       </c>
       <c r="D47" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>iPhone 15</t>
         </is>
       </c>
       <c r="E47" s="12" t="inlineStr">
@@ -2699,12 +2699,12 @@
       </c>
       <c r="C48" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Google Pixel 8</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
@@ -2750,12 +2750,12 @@
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D49" s="12" t="inlineStr">
         <is>
-          <t>Dell Latitude 7440</t>
+          <t>Samsung Galaxy S23 FE</t>
         </is>
       </c>
       <c r="E49" s="12" t="inlineStr">
@@ -2801,12 +2801,12 @@
       </c>
       <c r="C50" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>iPhone 14</t>
         </is>
       </c>
       <c r="E50" s="12" t="str"/>
@@ -2895,12 +2895,12 @@
       </c>
       <c r="C52" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>iPhone 15</t>
         </is>
       </c>
       <c r="E52" s="12" t="str"/>
@@ -2942,12 +2942,12 @@
       </c>
       <c r="C53" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D53" s="12" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14</t>
+          <t>Google Pixel 8</t>
         </is>
       </c>
       <c r="E53" s="12" t="str"/>
@@ -2989,12 +2989,12 @@
       </c>
       <c r="C54" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>iPhone 14</t>
         </is>
       </c>
       <c r="E54" s="12" t="str"/>
@@ -3083,12 +3083,12 @@
       </c>
       <c r="C56" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>iPhone 15</t>
         </is>
       </c>
       <c r="E56" s="12" t="str"/>
@@ -3130,12 +3130,12 @@
       </c>
       <c r="C57" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D57" s="12" t="inlineStr">
         <is>
-          <t>MacBook Pro 14</t>
+          <t>Google Pixel 8</t>
         </is>
       </c>
       <c r="E57" s="12" t="str"/>
@@ -3177,12 +3177,12 @@
       </c>
       <c r="C58" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Samsung Galaxy S23 FE</t>
         </is>
       </c>
       <c r="E58" s="12" t="str"/>
@@ -3229,7 +3229,7 @@
       </c>
       <c r="D59" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>iPhone 14</t>
         </is>
       </c>
       <c r="E59" s="12" t="str"/>
@@ -3271,12 +3271,12 @@
       </c>
       <c r="C60" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Samsung Galaxy S24</t>
         </is>
       </c>
       <c r="E60" s="12" t="str"/>
@@ -3318,12 +3318,12 @@
       </c>
       <c r="C61" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D61" s="12" t="inlineStr">
         <is>
-          <t>Dell Latitude 7440</t>
+          <t>iPhone 15</t>
         </is>
       </c>
       <c r="E61" s="12" t="str"/>
@@ -3365,12 +3365,12 @@
       </c>
       <c r="C62" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Google Pixel 8</t>
         </is>
       </c>
       <c r="E62" s="12" t="inlineStr">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="D63" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Samsung Galaxy S23 FE</t>
         </is>
       </c>
       <c r="E63" s="12" t="inlineStr">
@@ -3467,12 +3467,12 @@
       </c>
       <c r="C64" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Samsung Galaxy S24</t>
         </is>
       </c>
       <c r="E64" s="12" t="inlineStr">
@@ -3518,12 +3518,12 @@
       </c>
       <c r="C65" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D65" s="12" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14</t>
+          <t>iPhone 15</t>
         </is>
       </c>
       <c r="E65" s="12" t="inlineStr">
@@ -3569,12 +3569,12 @@
       </c>
       <c r="C66" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Google Pixel 8</t>
         </is>
       </c>
       <c r="E66" s="12" t="inlineStr">
@@ -3625,7 +3625,7 @@
       </c>
       <c r="D67" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Samsung Galaxy S23 FE</t>
         </is>
       </c>
       <c r="E67" s="12" t="inlineStr">
@@ -3671,12 +3671,12 @@
       </c>
       <c r="C68" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>iPhone 14</t>
         </is>
       </c>
       <c r="E68" s="12" t="inlineStr">
@@ -3722,12 +3722,12 @@
       </c>
       <c r="C69" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D69" s="12" t="inlineStr">
         <is>
-          <t>MacBook Pro 14</t>
+          <t>Samsung Galaxy S24</t>
         </is>
       </c>
       <c r="E69" s="12" t="inlineStr">
@@ -3773,12 +3773,12 @@
       </c>
       <c r="C70" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>iPhone 15</t>
         </is>
       </c>
       <c r="E70" s="12" t="inlineStr">
@@ -3829,7 +3829,7 @@
       </c>
       <c r="D71" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Google Pixel 8</t>
         </is>
       </c>
       <c r="E71" s="12" t="inlineStr">
@@ -3875,12 +3875,12 @@
       </c>
       <c r="C72" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Samsung Galaxy S23 FE</t>
         </is>
       </c>
       <c r="E72" s="12" t="inlineStr">
@@ -3926,12 +3926,12 @@
       </c>
       <c r="C73" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D73" s="12" t="inlineStr">
         <is>
-          <t>Dell Latitude 7440</t>
+          <t>iPhone 14</t>
         </is>
       </c>
       <c r="E73" s="12" t="inlineStr">
@@ -3977,12 +3977,12 @@
       </c>
       <c r="C74" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Mobile Device</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>iPhone 15</t>
         </is>
       </c>
       <c r="E74" s="12" t="inlineStr">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="D75" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Google Pixel 8</t>
         </is>
       </c>
       <c r="E75" s="12" t="inlineStr">
@@ -4084,7 +4084,7 @@
       </c>
       <c r="D76" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Fortinet FortiSwitch 148F</t>
         </is>
       </c>
       <c r="E76" s="12" t="inlineStr">
@@ -4130,12 +4130,12 @@
       </c>
       <c r="C77" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D77" s="12" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14</t>
+          <t>Cisco C9300</t>
         </is>
       </c>
       <c r="E77" s="12" t="inlineStr">
@@ -4181,12 +4181,12 @@
       </c>
       <c r="C78" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Aruba 6300M</t>
         </is>
       </c>
       <c r="E78" s="12" t="inlineStr">
@@ -4232,12 +4232,12 @@
       </c>
       <c r="C79" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D79" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Juniper EX3400</t>
         </is>
       </c>
       <c r="E79" s="12" t="inlineStr">
@@ -4288,7 +4288,7 @@
       </c>
       <c r="D80" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Cisco Meraki MS250</t>
         </is>
       </c>
       <c r="E80" s="12" t="inlineStr">
@@ -4334,12 +4334,12 @@
       </c>
       <c r="C81" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D81" s="12" t="inlineStr">
         <is>
-          <t>MacBook Pro 14</t>
+          <t>Fortinet FortiSwitch 148F</t>
         </is>
       </c>
       <c r="E81" s="12" t="inlineStr">
@@ -4385,12 +4385,12 @@
       </c>
       <c r="C82" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Cisco C9300</t>
         </is>
       </c>
       <c r="E82" s="12" t="inlineStr">
@@ -4436,12 +4436,12 @@
       </c>
       <c r="C83" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D83" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Aruba 6300M</t>
         </is>
       </c>
       <c r="E83" s="12" t="inlineStr">
@@ -4492,7 +4492,7 @@
       </c>
       <c r="D84" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Cisco Meraki MS250</t>
         </is>
       </c>
       <c r="E84" s="12" t="inlineStr">
@@ -4538,12 +4538,12 @@
       </c>
       <c r="C85" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D85" s="12" t="inlineStr">
         <is>
-          <t>Dell Latitude 7440</t>
+          <t>Fortinet FortiSwitch 148F</t>
         </is>
       </c>
       <c r="E85" s="12" t="inlineStr">
@@ -4589,12 +4589,12 @@
       </c>
       <c r="C86" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Cisco C9300</t>
         </is>
       </c>
       <c r="E86" s="12" t="inlineStr">
@@ -4640,12 +4640,12 @@
       </c>
       <c r="C87" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D87" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Aruba 6300M</t>
         </is>
       </c>
       <c r="E87" s="12" t="inlineStr">
@@ -4696,7 +4696,7 @@
       </c>
       <c r="D88" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Juniper EX3400</t>
         </is>
       </c>
       <c r="E88" s="12" t="inlineStr">
@@ -4742,12 +4742,12 @@
       </c>
       <c r="C89" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D89" s="12" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14</t>
+          <t>Cisco Meraki MS250</t>
         </is>
       </c>
       <c r="E89" s="12" t="inlineStr">
@@ -4793,12 +4793,12 @@
       </c>
       <c r="C90" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Fortinet FortiSwitch 148F</t>
         </is>
       </c>
       <c r="E90" s="12" t="inlineStr">
@@ -4844,12 +4844,12 @@
       </c>
       <c r="C91" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D91" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Cisco C9300</t>
         </is>
       </c>
       <c r="E91" s="12" t="inlineStr">
@@ -4900,7 +4900,7 @@
       </c>
       <c r="D92" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Aruba 6300M</t>
         </is>
       </c>
       <c r="E92" s="12" t="inlineStr">
@@ -4946,12 +4946,12 @@
       </c>
       <c r="C93" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D93" s="12" t="inlineStr">
         <is>
-          <t>MacBook Pro 14</t>
+          <t>Juniper EX3400</t>
         </is>
       </c>
       <c r="E93" s="12" t="inlineStr">
@@ -4997,12 +4997,12 @@
       </c>
       <c r="C94" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Fortinet FortiSwitch 148F</t>
         </is>
       </c>
       <c r="E94" s="12" t="inlineStr">
@@ -5048,12 +5048,12 @@
       </c>
       <c r="C95" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D95" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Cisco C9300</t>
         </is>
       </c>
       <c r="E95" s="12" t="inlineStr">
@@ -5104,7 +5104,7 @@
       </c>
       <c r="D96" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Aruba 6300M</t>
         </is>
       </c>
       <c r="E96" s="12" t="inlineStr">
@@ -5150,12 +5150,12 @@
       </c>
       <c r="C97" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D97" s="12" t="inlineStr">
         <is>
-          <t>Dell Latitude 7440</t>
+          <t>Juniper EX3400</t>
         </is>
       </c>
       <c r="E97" s="12" t="inlineStr">
@@ -5201,12 +5201,12 @@
       </c>
       <c r="C98" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Cisco Meraki MS250</t>
         </is>
       </c>
       <c r="E98" s="12" t="inlineStr">
@@ -5252,12 +5252,12 @@
       </c>
       <c r="C99" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D99" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Fortinet FortiSwitch 148F</t>
         </is>
       </c>
       <c r="E99" s="12" t="inlineStr">
@@ -5354,12 +5354,12 @@
       </c>
       <c r="C101" s="12" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D101" s="12" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14</t>
+          <t>Aruba 6300M</t>
         </is>
       </c>
       <c r="E101" s="12" t="inlineStr">
@@ -5405,12 +5405,12 @@
       </c>
       <c r="C102" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Juniper EX3400</t>
         </is>
       </c>
       <c r="E102" s="12" t="inlineStr">
@@ -5456,12 +5456,12 @@
       </c>
       <c r="C103" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Network Asset</t>
         </is>
       </c>
       <c r="D103" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Cisco Meraki MS250</t>
         </is>
       </c>
       <c r="E103" s="12" t="inlineStr">
@@ -5507,12 +5507,12 @@
       </c>
       <c r="C104" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>HP EliteBook 840 G10</t>
         </is>
       </c>
       <c r="E104" s="12" t="inlineStr">
@@ -5563,7 +5563,7 @@
       </c>
       <c r="D105" s="12" t="inlineStr">
         <is>
-          <t>MacBook Pro 14</t>
+          <t>Microsoft Surface Laptop 5</t>
         </is>
       </c>
       <c r="E105" s="12" t="inlineStr">
@@ -5609,12 +5609,12 @@
       </c>
       <c r="C106" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Lenovo ThinkPad X1 Carbon</t>
         </is>
       </c>
       <c r="E106" s="12" t="inlineStr">
@@ -5660,12 +5660,12 @@
       </c>
       <c r="C107" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D107" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Lenovo ThinkPad T14</t>
         </is>
       </c>
       <c r="E107" s="12" t="inlineStr">
@@ -5711,12 +5711,12 @@
       </c>
       <c r="C108" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>MacBook Pro 14</t>
         </is>
       </c>
       <c r="E108" s="12" t="inlineStr">
@@ -5813,12 +5813,12 @@
       </c>
       <c r="C110" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>HP EliteBook 840 G10</t>
         </is>
       </c>
       <c r="E110" s="12" t="inlineStr">
@@ -5864,12 +5864,12 @@
       </c>
       <c r="C111" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D111" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Microsoft Surface Laptop 5</t>
         </is>
       </c>
       <c r="E111" s="12" t="inlineStr">
@@ -5915,12 +5915,12 @@
       </c>
       <c r="C112" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Lenovo ThinkPad X1 Carbon</t>
         </is>
       </c>
       <c r="E112" s="12" t="inlineStr">
@@ -6017,12 +6017,12 @@
       </c>
       <c r="C114" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D114" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Dell Latitude 7440</t>
         </is>
       </c>
       <c r="E114" s="12" t="inlineStr">
@@ -6068,12 +6068,12 @@
       </c>
       <c r="C115" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D115" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>HP EliteBook 840 G10</t>
         </is>
       </c>
       <c r="E115" s="12" t="inlineStr">
@@ -6119,12 +6119,12 @@
       </c>
       <c r="C116" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D116" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Microsoft Surface Laptop 5</t>
         </is>
       </c>
       <c r="E116" s="12" t="inlineStr">
@@ -6175,7 +6175,7 @@
       </c>
       <c r="D117" s="12" t="inlineStr">
         <is>
-          <t>MacBook Pro 14</t>
+          <t>Lenovo ThinkPad X1 Carbon</t>
         </is>
       </c>
       <c r="E117" s="12" t="inlineStr">
@@ -6221,12 +6221,12 @@
       </c>
       <c r="C118" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D118" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Lenovo ThinkPad T14</t>
         </is>
       </c>
       <c r="E118" s="12" t="inlineStr">
@@ -6272,12 +6272,12 @@
       </c>
       <c r="C119" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D119" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>MacBook Pro 14</t>
         </is>
       </c>
       <c r="E119" s="12" t="inlineStr">
@@ -6323,12 +6323,12 @@
       </c>
       <c r="C120" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D120" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Dell Latitude 7440</t>
         </is>
       </c>
       <c r="E120" s="12" t="inlineStr">
@@ -6379,7 +6379,7 @@
       </c>
       <c r="D121" s="12" t="inlineStr">
         <is>
-          <t>Dell Latitude 7440</t>
+          <t>HP EliteBook 840 G10</t>
         </is>
       </c>
       <c r="E121" s="12" t="inlineStr">
@@ -6425,12 +6425,12 @@
       </c>
       <c r="C122" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D122" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Microsoft Surface Laptop 5</t>
         </is>
       </c>
       <c r="E122" s="12" t="inlineStr">
@@ -6476,12 +6476,12 @@
       </c>
       <c r="C123" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D123" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Lenovo ThinkPad X1 Carbon</t>
         </is>
       </c>
       <c r="E123" s="12" t="inlineStr">
@@ -6527,12 +6527,12 @@
       </c>
       <c r="C124" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D124" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>MacBook Pro 14</t>
         </is>
       </c>
       <c r="E124" s="12" t="inlineStr">
@@ -6583,7 +6583,7 @@
       </c>
       <c r="D125" s="12" t="inlineStr">
         <is>
-          <t>Lenovo ThinkPad T14</t>
+          <t>Dell Latitude 7440</t>
         </is>
       </c>
       <c r="E125" s="12" t="str"/>
@@ -6625,12 +6625,12 @@
       </c>
       <c r="C126" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D126" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>HP EliteBook 840 G10</t>
         </is>
       </c>
       <c r="E126" s="12" t="str"/>
@@ -6672,12 +6672,12 @@
       </c>
       <c r="C127" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D127" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Microsoft Surface Laptop 5</t>
         </is>
       </c>
       <c r="E127" s="12" t="str"/>
@@ -6719,12 +6719,12 @@
       </c>
       <c r="C128" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D128" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Lenovo ThinkPad X1 Carbon</t>
         </is>
       </c>
       <c r="E128" s="12" t="str"/>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="D129" s="12" t="inlineStr">
         <is>
-          <t>MacBook Pro 14</t>
+          <t>Lenovo ThinkPad T14</t>
         </is>
       </c>
       <c r="E129" s="12" t="str"/>
@@ -6813,12 +6813,12 @@
       </c>
       <c r="C130" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D130" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>MacBook Pro 14</t>
         </is>
       </c>
       <c r="E130" s="12" t="str"/>
@@ -6860,12 +6860,12 @@
       </c>
       <c r="C131" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D131" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>Dell Latitude 7440</t>
         </is>
       </c>
       <c r="E131" s="12" t="inlineStr">
@@ -6911,12 +6911,12 @@
       </c>
       <c r="C132" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D132" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>HP EliteBook 840 G10</t>
         </is>
       </c>
       <c r="E132" s="12" t="inlineStr">
@@ -6967,7 +6967,7 @@
       </c>
       <c r="D133" s="12" t="inlineStr">
         <is>
-          <t>Dell Latitude 7440</t>
+          <t>Microsoft Surface Laptop 5</t>
         </is>
       </c>
       <c r="E133" s="12" t="inlineStr">
@@ -7013,12 +7013,12 @@
       </c>
       <c r="C134" s="12" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D134" s="12" t="inlineStr">
         <is>
-          <t>Dell U2723QE</t>
+          <t>Lenovo ThinkPad T14</t>
         </is>
       </c>
       <c r="E134" s="12" t="inlineStr">
@@ -7064,12 +7064,12 @@
       </c>
       <c r="C135" s="12" t="inlineStr">
         <is>
-          <t>Mobile Device</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D135" s="12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S24</t>
+          <t>MacBook Pro 14</t>
         </is>
       </c>
       <c r="E135" s="12" t="inlineStr">
@@ -7115,12 +7115,12 @@
       </c>
       <c r="C136" s="12" t="inlineStr">
         <is>
-          <t>Network Asset</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="D136" s="12" t="inlineStr">
         <is>
-          <t>Cisco C9300</t>
+          <t>Dell Latitude 7440</t>
         </is>
       </c>
       <c r="E136" s="12" t="inlineStr">

</xml_diff>